<commit_message>
CI Reports [2026-07-01 18:05]: Login — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report_Git/Feature Reports/Login.xlsx
+++ b/Test Execution Report_Git/Feature Reports/Login.xlsx
@@ -1440,10 +1440,10 @@
         <v>SQL injection in password rejected; authentication not bypassed; stays on /Account/Login; no SQL error</v>
       </c>
       <c r="K19" t="str">
-        <v>All assertions passed via Playwright</v>
+        <v>Error: expect(page).toHaveURL(expected) failed Expected pattern: /Login/ Received string: "" Timeout: 5000ms Call log: - Expect "toHaveURL" with timeout 5000ms - waiting for navigation to finish...</v>
       </c>
       <c r="L19" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="M19" t="str">
         <v>Playwright Automation</v>
@@ -1647,6 +1647,58 @@
         <v>Remarks</v>
       </c>
     </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str">
+        <v>BUG-LOGIN-001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>SQL injection in password handled safely</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D2" t="str">
+        <v>TC-LOGIN-018</v>
+      </c>
+      <c r="E2" t="str">
+        <v>High</v>
+      </c>
+      <c r="F2" t="str">
+        <v>P2</v>
+      </c>
+      <c r="G2" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="H2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Enter sajith_xyz + ' OR '1'='1 as password
+2. Click Sign In
+3. Check URL and auth state for SQL bypass</v>
+      </c>
+      <c r="I2" t="str">
+        <v>SQL injection in password rejected; authentication not bypassed; stays on /Account/Login; no SQL error</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Error: expect(page).toHaveURL(expected) failed Expected pattern: /Login/ Received string: "" Timeout: 5000ms Call log: - Expect "toHaveURL" with timeout 5000ms - waiting for navigation to finish...</v>
+      </c>
+      <c r="K2" t="str">
+        <v>New</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="M2" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v>Not Run</v>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:P2"/>

</xml_diff>

<commit_message>
CI Reports [2026-07-01 18:43]: Login — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report_Git/Feature Reports/Login.xlsx
+++ b/Test Execution Report_Git/Feature Reports/Login.xlsx
@@ -1440,7 +1440,7 @@
         <v>SQL injection in password rejected; authentication not bypassed; stays on /Account/Login; no SQL error</v>
       </c>
       <c r="K19" t="str">
-        <v>Error: expect(page).toHaveURL(expected) failed Expected pattern: /Login/ Received string: "" Timeout: 5000ms Call log: - Expect "toHaveURL" with timeout 5000ms - waiting for navigation to finish...</v>
+        <v>Error: expect(page).toHaveURL(expected) failed Expected pattern: /Login/ Received string: "" Timeout: 5000ms Call log: - Expect "toHaveURL" with timeout 5000ms - waiting for" http://customerportal.dev-ts.online/Account/Login" navigation to finish...</v>
       </c>
       <c r="L19" t="str">
         <v>FAIL</v>
@@ -1678,7 +1678,7 @@
         <v>SQL injection in password rejected; authentication not bypassed; stays on /Account/Login; no SQL error</v>
       </c>
       <c r="J2" t="str">
-        <v>Error: expect(page).toHaveURL(expected) failed Expected pattern: /Login/ Received string: "" Timeout: 5000ms Call log: - Expect "toHaveURL" with timeout 5000ms - waiting for navigation to finish...</v>
+        <v>Error: expect(page).toHaveURL(expected) failed Expected pattern: /Login/ Received string: "" Timeout: 5000ms Call log: - Expect "toHaveURL" with timeout 5000ms - waiting for" http://customerportal.dev-ts.online/Account/Login" navigation to finish...</v>
       </c>
       <c r="K2" t="str">
         <v>New</v>

</xml_diff>